<commit_message>
Added screenshots to README
</commit_message>
<xml_diff>
--- a/Attendance_Report.xlsx
+++ b/Attendance_Report.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,17 +451,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Akshaya D</t>
+          <t>Akshaya</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>09:26:06</t>
+          <t>15:39:05</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -483,12 +483,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>11:26:16</t>
+          <t>14:18:12</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -510,15 +510,150 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>22:36:00</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Akshaya</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>20:28:00</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Akshaya</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>21:21:51</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Akshaya D</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>09:26:06</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Akshaya</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>11:26:16</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Akshaya</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>15:49:04</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>Present</t>
         </is>

</xml_diff>